<commit_message>
que los datos los tome del excel
</commit_message>
<xml_diff>
--- a/reports/banrep.xlsx
+++ b/reports/banrep.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t xml:space="preserve">Fecha</t>
   </si>
@@ -140,6 +140,27 @@
   </si>
   <si>
     <t xml:space="preserve">2026-07-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-15</t>
   </si>
 </sst>
 </file>
@@ -237,16 +258,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -442,532 +467,632 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="1" t="n">
         <v>488</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="1" t="n">
         <v>4033</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>1662</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>770</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>5525</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>1893</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>770</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="1" t="n">
         <v>5525</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>1893</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>923</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="1" t="n">
         <v>6233</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>2083</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="1" t="n">
         <v>56</v>
       </c>
-      <c r="C6" s="0" t="n">
+      <c r="C6" s="1" t="n">
         <v>729</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>161</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <v>102</v>
       </c>
-      <c r="C7" s="0" t="n">
+      <c r="C7" s="1" t="n">
         <v>1855</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="D7" s="1" t="n">
         <v>372</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="1" t="n">
         <v>1415</v>
       </c>
-      <c r="C8" s="0" t="n">
+      <c r="C8" s="1" t="n">
         <v>3552</v>
       </c>
-      <c r="D8" s="0" t="n">
+      <c r="D8" s="1" t="n">
         <v>660</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="1" t="n">
         <v>19890</v>
       </c>
-      <c r="C9" s="0" t="n">
+      <c r="C9" s="1" t="n">
         <v>4615</v>
       </c>
-      <c r="D9" s="0" t="n">
+      <c r="D9" s="1" t="n">
         <v>1323</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="1" t="n">
         <v>26704</v>
       </c>
-      <c r="C10" s="0" t="n">
+      <c r="C10" s="1" t="n">
         <v>5671</v>
       </c>
-      <c r="D10" s="0" t="n">
+      <c r="D10" s="1" t="n">
         <v>1576</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="1" t="n">
         <v>29937</v>
       </c>
-      <c r="C11" s="0" t="n">
+      <c r="C11" s="1" t="n">
         <v>7463</v>
       </c>
-      <c r="D11" s="0" t="n">
+      <c r="D11" s="1" t="n">
         <v>1843</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="1" t="n">
         <v>31036</v>
       </c>
-      <c r="C12" s="0" t="n">
+      <c r="C12" s="1" t="n">
         <v>8124</v>
       </c>
-      <c r="D12" s="0" t="n">
+      <c r="D12" s="1" t="n">
         <v>2158</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="1" t="n">
         <v>1595</v>
       </c>
-      <c r="C13" s="0" t="n">
+      <c r="C13" s="1" t="n">
         <v>601</v>
       </c>
-      <c r="D13" s="0" t="n">
+      <c r="D13" s="1" t="n">
         <v>205</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="1" t="n">
         <v>9020</v>
       </c>
-      <c r="C14" s="0" t="n">
+      <c r="C14" s="1" t="n">
         <v>1240</v>
       </c>
-      <c r="D14" s="0" t="n">
+      <c r="D14" s="1" t="n">
         <v>472</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="0" t="n">
+      <c r="B15" s="1" t="n">
         <v>29765</v>
       </c>
-      <c r="C15" s="0" t="n">
+      <c r="C15" s="1" t="n">
         <v>2924</v>
       </c>
-      <c r="D15" s="0" t="n">
+      <c r="D15" s="1" t="n">
         <v>895</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="0" t="n">
+      <c r="B16" s="1" t="n">
         <v>33115</v>
       </c>
-      <c r="C16" s="0" t="n">
+      <c r="C16" s="1" t="n">
         <v>4607</v>
       </c>
-      <c r="D16" s="0" t="n">
+      <c r="D16" s="1" t="n">
         <v>1142</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="0" t="n">
+      <c r="B17" s="1" t="n">
         <v>36890</v>
       </c>
-      <c r="C17" s="0" t="n">
+      <c r="C17" s="1" t="n">
         <v>5640</v>
       </c>
-      <c r="D17" s="0" t="n">
+      <c r="D17" s="1" t="n">
         <v>1347</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" s="1" t="n">
         <v>39235</v>
       </c>
-      <c r="C18" s="0" t="n">
+      <c r="C18" s="1" t="n">
         <v>6626</v>
       </c>
-      <c r="D18" s="0" t="n">
+      <c r="D18" s="1" t="n">
         <v>1699</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="1" t="n">
         <v>43204</v>
       </c>
-      <c r="C19" s="0" t="n">
+      <c r="C19" s="1" t="n">
         <v>7594</v>
       </c>
-      <c r="D19" s="0" t="n">
+      <c r="D19" s="1" t="n">
         <v>1930</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" s="1" t="n">
         <v>3556</v>
       </c>
-      <c r="C20" s="0" t="n">
+      <c r="C20" s="1" t="n">
         <v>787</v>
       </c>
-      <c r="D20" s="0" t="n">
+      <c r="D20" s="1" t="n">
         <v>238</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" s="1" t="n">
         <v>8490</v>
       </c>
-      <c r="C21" s="0" t="n">
+      <c r="C21" s="1" t="n">
         <v>2261</v>
       </c>
-      <c r="D21" s="0" t="n">
+      <c r="D21" s="1" t="n">
         <v>527</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" s="1" t="n">
         <v>21937</v>
       </c>
-      <c r="C22" s="0" t="n">
+      <c r="C22" s="1" t="n">
         <v>4297</v>
       </c>
-      <c r="D22" s="0" t="n">
+      <c r="D22" s="1" t="n">
         <v>743</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="0" t="n">
+      <c r="B23" s="1" t="n">
         <v>28919</v>
       </c>
-      <c r="C23" s="0" t="n">
+      <c r="C23" s="1" t="n">
         <v>6563</v>
       </c>
-      <c r="D23" s="0" t="n">
+      <c r="D23" s="1" t="n">
         <v>953</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="0" t="n">
+      <c r="B24" s="1" t="n">
         <v>38219</v>
       </c>
-      <c r="C24" s="0" t="n">
+      <c r="C24" s="1" t="n">
         <v>7716</v>
       </c>
-      <c r="D24" s="0" t="n">
+      <c r="D24" s="1" t="n">
         <v>1250</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="0" t="n">
+      <c r="B25" s="1" t="n">
         <v>39241</v>
       </c>
-      <c r="C25" s="0" t="n">
+      <c r="C25" s="1" t="n">
         <v>8475</v>
       </c>
-      <c r="D25" s="0" t="n">
+      <c r="D25" s="1" t="n">
         <v>1511</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="0" t="n">
+      <c r="B26" s="1" t="n">
         <v>39955</v>
       </c>
-      <c r="C26" s="0" t="n">
+      <c r="C26" s="1" t="n">
         <v>9973</v>
       </c>
-      <c r="D26" s="0" t="n">
+      <c r="D26" s="1" t="n">
         <v>1711</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B27" s="0" t="n">
+      <c r="B27" s="1" t="n">
         <v>2225</v>
       </c>
-      <c r="C27" s="0" t="n">
+      <c r="C27" s="1" t="n">
         <v>1171</v>
       </c>
-      <c r="D27" s="0" t="n">
+      <c r="D27" s="1" t="n">
         <v>185</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="0" t="n">
+      <c r="B28" s="1" t="n">
         <v>3896</v>
       </c>
-      <c r="C28" s="0" t="n">
+      <c r="C28" s="1" t="n">
         <v>2544</v>
       </c>
-      <c r="D28" s="0" t="n">
+      <c r="D28" s="1" t="n">
         <v>1060</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="A29" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B29" s="0" t="n">
+      <c r="B29" s="1" t="n">
         <v>6462</v>
       </c>
-      <c r="C29" s="0" t="n">
+      <c r="C29" s="1" t="n">
         <v>3907</v>
       </c>
-      <c r="D29" s="0" t="n">
+      <c r="D29" s="1" t="n">
         <v>1281</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="0" t="n">
+      <c r="B30" s="1" t="n">
         <v>8079</v>
       </c>
-      <c r="C30" s="0" t="n">
+      <c r="C30" s="1" t="n">
         <v>5711</v>
       </c>
-      <c r="D30" s="0" t="n">
+      <c r="D30" s="1" t="n">
         <v>1496</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B31" s="0" t="n">
+      <c r="B31" s="1" t="n">
         <v>11459</v>
       </c>
-      <c r="C31" s="0" t="n">
+      <c r="C31" s="1" t="n">
         <v>7224</v>
       </c>
-      <c r="D31" s="2" t="n">
+      <c r="D31" s="3" t="n">
         <v>1661</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+      <c r="A32" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B32" s="0" t="n">
+      <c r="B32" s="1" t="n">
         <v>13392</v>
       </c>
-      <c r="C32" s="0" t="n">
+      <c r="C32" s="1" t="n">
         <v>8441</v>
       </c>
-      <c r="D32" s="0" t="n">
+      <c r="D32" s="1" t="n">
         <v>1838</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+      <c r="A33" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="0" t="n">
+      <c r="B33" s="1" t="n">
         <v>14756</v>
       </c>
-      <c r="C33" s="0" t="n">
+      <c r="C33" s="1" t="n">
         <v>9375</v>
       </c>
-      <c r="D33" s="0" t="n">
+      <c r="D33" s="1" t="n">
         <v>2134</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+      <c r="A34" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="0" t="n">
+      <c r="B34" s="1" t="n">
         <v>1870</v>
       </c>
-      <c r="C34" s="0" t="n">
+      <c r="C34" s="1" t="n">
         <v>1312</v>
       </c>
-      <c r="D34" s="0" t="n">
+      <c r="D34" s="1" t="n">
         <v>213</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="A35" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B35" s="0" t="n">
+      <c r="B35" s="1" t="n">
         <v>3755</v>
       </c>
-      <c r="C35" s="0" t="n">
+      <c r="C35" s="1" t="n">
         <v>2663</v>
       </c>
-      <c r="D35" s="0" t="n">
+      <c r="D35" s="1" t="n">
         <v>433</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
+      <c r="A36" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="0" t="n">
+      <c r="B36" s="1" t="n">
         <v>6540</v>
       </c>
-      <c r="C36" s="0" t="n">
+      <c r="C36" s="1" t="n">
         <v>4051</v>
       </c>
-      <c r="D36" s="0" t="n">
+      <c r="D36" s="1" t="n">
         <v>645</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+      <c r="A37" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B37" s="0" t="n">
+      <c r="B37" s="1" t="n">
         <v>9912</v>
       </c>
-      <c r="C37" s="0" t="n">
+      <c r="C37" s="1" t="n">
         <v>5590</v>
       </c>
-      <c r="D37" s="0" t="n">
+      <c r="D37" s="1" t="n">
         <v>1006</v>
       </c>
     </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>14462</v>
+      </c>
+      <c r="C38" s="1" t="n">
+        <v>8624</v>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>1256</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>16642</v>
+      </c>
+      <c r="C39" s="1" t="n">
+        <v>10060</v>
+      </c>
+      <c r="D39" s="1" t="n">
+        <v>1477</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>18966</v>
+      </c>
+      <c r="C40" s="1" t="n">
+        <v>10913</v>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>1686</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>820</v>
+      </c>
+      <c r="C41" s="1" t="n">
+        <v>397</v>
+      </c>
+      <c r="D41" s="1" t="n">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>1268</v>
+      </c>
+      <c r="C42" s="1" t="n">
+        <v>1001</v>
+      </c>
+      <c r="D42" s="1" t="n">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>8414</v>
+      </c>
+      <c r="C43" s="1" t="n">
+        <v>2602</v>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>56398</v>
+      </c>
+      <c r="C44" s="1" t="n">
+        <v>4320</v>
+      </c>
+      <c r="D44" s="1" t="n">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>